<commit_message>
Reponer stock con stock detallado
</commit_message>
<xml_diff>
--- a/reportes/reporte_stock.xlsx
+++ b/reportes/reporte_stock.xlsx
@@ -450,13 +450,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
         <v>889</v>
       </c>
       <c r="D2" t="n">
-        <v>66675</v>
+        <v>47117</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -471,13 +471,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="C3" t="n">
         <v>666</v>
       </c>
       <c r="D3" t="n">
-        <v>60606</v>
+        <v>40626</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="C4" t="n">
         <v>1778</v>
       </c>
       <c r="D4" t="n">
-        <v>128016</v>
+        <v>46228</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -513,13 +513,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="C5" t="n">
         <v>1630</v>
       </c>
       <c r="D5" t="n">
-        <v>140180</v>
+        <v>104320</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -534,13 +534,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="C6" t="n">
         <v>740</v>
       </c>
       <c r="D6" t="n">
-        <v>68820</v>
+        <v>48840</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="C7" t="n">
         <v>518</v>
       </c>
       <c r="D7" t="n">
-        <v>28490</v>
+        <v>15540</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C8" t="n">
         <v>666</v>
       </c>
       <c r="D8" t="n">
-        <v>29304</v>
+        <v>24642</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -597,13 +597,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C9" t="n">
         <v>370</v>
       </c>
       <c r="D9" t="n">
-        <v>18870</v>
+        <v>24790</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -618,13 +618,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>97</v>
+        <v>45</v>
       </c>
       <c r="C10" t="n">
         <v>2222</v>
       </c>
       <c r="D10" t="n">
-        <v>215534</v>
+        <v>99990</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -639,13 +639,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C11" t="n">
         <v>1037</v>
       </c>
       <c r="D11" t="n">
-        <v>66368</v>
+        <v>65331</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -660,13 +660,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="C12" t="n">
         <v>296</v>
       </c>
       <c r="D12" t="n">
-        <v>29304</v>
+        <v>14208</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -681,13 +681,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="C13" t="n">
         <v>1481</v>
       </c>
       <c r="D13" t="n">
-        <v>118480</v>
+        <v>74050</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="C14" t="n">
         <v>1407</v>
       </c>
       <c r="D14" t="n">
-        <v>95676</v>
+        <v>53466</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,13 +723,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="C15" t="n">
         <v>1333</v>
       </c>
       <c r="D15" t="n">
-        <v>111972</v>
+        <v>41323</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -744,13 +744,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="C16" t="n">
         <v>889</v>
       </c>
       <c r="D16" t="n">
-        <v>85344</v>
+        <v>43561</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -765,13 +765,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="C17" t="n">
         <v>815</v>
       </c>
       <c r="D17" t="n">
-        <v>72535</v>
+        <v>44825</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -786,13 +786,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="C18" t="n">
         <v>1185</v>
       </c>
       <c r="D18" t="n">
-        <v>111390</v>
+        <v>61620</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -807,13 +807,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C19" t="n">
         <v>666</v>
       </c>
       <c r="D19" t="n">
-        <v>31302</v>
+        <v>39294</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Entrega y direccion, eliminacion de pandas y tabulate
</commit_message>
<xml_diff>
--- a/reportes/reporte_stock.xlsx
+++ b/reportes/reporte_stock.xlsx
@@ -486,13 +486,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1050</v>
+        <v>1037</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45150</v>
+        <v>66368</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>675</v>
+        <v>666</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>32400</v>
+        <v>39294</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>23625</v>
+        <v>12950</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -549,13 +549,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1500</v>
+        <v>1481</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>94500</v>
+        <v>51835</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -570,13 +570,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>525</v>
+        <v>518</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>28875</v>
+        <v>25900</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -591,13 +591,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1200</v>
+        <v>1185</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>74400</v>
+        <v>71100</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -612,13 +612,13 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>900</v>
+        <v>889</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>35100</v>
+        <v>33782</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -633,13 +633,13 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>825</v>
+        <v>814</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>30525</v>
+        <v>56980</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1650</v>
+        <v>1629</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>64350</v>
+        <v>55386</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1425</v>
+        <v>1407</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>84075</v>
+        <v>75978</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -696,13 +696,13 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>750</v>
+        <v>740</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>40500</v>
+        <v>42920</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1800</v>
+        <v>1778</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>122400</v>
+        <v>58674</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1350</v>
+        <v>1333</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>75600</v>
+        <v>59985</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2250</v>
+        <v>2222</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>74250</v>
+        <v>119988</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>675</v>
+        <v>666</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>21600</v>
+        <v>34632</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>15300</v>
+        <v>17168</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>675</v>
+        <v>666</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>28350</v>
+        <v>31302</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>900</v>
+        <v>889</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>39600</v>
+        <v>62230</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
agrega detalles al menu y mas opciones en el menu principal
</commit_message>
<xml_diff>
--- a/reportes/reporte_stock.xlsx
+++ b/reportes/reporte_stock.xlsx
@@ -486,13 +486,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>1037</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>66368</v>
+        <v>45628</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>666</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>39294</v>
+        <v>31968</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>370</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>12950</v>
+        <v>22940</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -549,13 +549,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>1481</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>51835</v>
+        <v>77012</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -570,13 +570,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>518</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>25900</v>
+        <v>25382</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -591,13 +591,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>1185</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>71100</v>
+        <v>50955</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -612,13 +612,13 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>889</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>33782</v>
+        <v>54229</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -633,13 +633,13 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>814</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>56980</v>
+        <v>43956</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>1629</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>55386</v>
+        <v>76563</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>1407</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>75978</v>
+        <v>98490</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -696,13 +696,13 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>740</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>42920</v>
+        <v>23680</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>1778</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>58674</v>
+        <v>78232</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>1333</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>59985</v>
+        <v>89311</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>2222</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>119988</v>
+        <v>153318</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>666</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>34632</v>
+        <v>42624</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>296</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>17168</v>
+        <v>13320</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>666</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>31302</v>
+        <v>37962</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>889</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>62230</v>
+        <v>45339</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Anotaciones en todos los archivos
</commit_message>
<xml_diff>
--- a/reportes/reporte_stock.xlsx
+++ b/reportes/reporte_stock.xlsx
@@ -486,13 +486,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>1046</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>58576</v>
+        <v>71128</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>672</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>21504</v>
+        <v>27552</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>373</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13801</v>
+        <v>20888</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -549,13 +549,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>1495</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>73255</v>
+        <v>94185</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -570,13 +570,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>523</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>19874</v>
+        <v>34518</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -591,13 +591,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>1196</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>78936</v>
+        <v>74152</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -612,13 +612,13 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>897</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>54717</v>
+        <v>37674</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -633,13 +633,13 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>822</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>41100</v>
+        <v>48498</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>1644</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>93708</v>
+        <v>115080</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>1420</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>69580</v>
+        <v>42600</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -696,13 +696,13 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>747</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>42579</v>
+        <v>46314</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>1794</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>75348</v>
+        <v>73554</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>1345</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>43040</v>
+        <v>94150</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>2242</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>69502</v>
+        <v>114342</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>672</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>24864</v>
+        <v>24192</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>299</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>15249</v>
+        <v>11661</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>672</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>26208</v>
+        <v>31584</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>897</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>38571</v>
+        <v>27807</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>

</xml_diff>